<commit_message>
adding find and replace, advanced sorting
</commit_message>
<xml_diff>
--- a/Excel/29_Find_and_Replace/Pinterest_Find_Replace_Practice.xlsx
+++ b/Excel/29_Find_and_Replace/Pinterest_Find_Replace_Practice.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Pinterest-Analytics-Project\Excel\29_Find_and_Replace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F51FFC3C-BA7B-4326-997F-53D0FA68C520}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9EEC6E1-FBC3-471D-947B-CFAAF41FF126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B7B0EF28-BA75-45B3-9BD8-ECED1051200E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{B7B0EF28-BA75-45B3-9BD8-ECED1051200E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="pin_data" sheetId="1" r:id="rId1"/>
+    <sheet name="find and replace_practice" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,9 +36,68 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="18">
+  <si>
+    <t>Pin Name</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Impressions</t>
+  </si>
+  <si>
+    <t>Engagement</t>
+  </si>
+  <si>
+    <t>Kitchen Storage</t>
+  </si>
+  <si>
+    <t>Kitchen</t>
+  </si>
+  <si>
+    <t>Handbag Fashion</t>
+  </si>
+  <si>
+    <t>Fashion</t>
+  </si>
+  <si>
+    <t>Home Decor</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Beauty Self-Care</t>
+  </si>
+  <si>
+    <t>Beauty</t>
+  </si>
+  <si>
+    <t>Kitchen Storage Ideas</t>
+  </si>
+  <si>
+    <t>Desk Setup</t>
+  </si>
+  <si>
+    <t>Skincare Products</t>
+  </si>
+  <si>
+    <t>Home Decor ideas ideas</t>
+  </si>
+  <si>
+    <t>Kitchen Storage ideas</t>
+  </si>
+  <si>
+    <t>Kitchen Storage ideas Ideas</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -45,16 +105,48 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -62,12 +154,204 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +686,334 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2598ACCE-E811-4140-9CA8-70BB5DCB6102}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="4" width="18.6328125" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="15">
+        <v>76</v>
+      </c>
+      <c r="D2" s="16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="15">
+        <v>45</v>
+      </c>
+      <c r="D3" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="15">
+        <v>41</v>
+      </c>
+      <c r="D4" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="15">
+        <v>57</v>
+      </c>
+      <c r="D5" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="15">
+        <v>63</v>
+      </c>
+      <c r="D6" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="15">
+        <v>35</v>
+      </c>
+      <c r="D7" s="16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="15">
+        <v>23</v>
+      </c>
+      <c r="D8" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="15">
+        <v>52</v>
+      </c>
+      <c r="D9" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="15">
+        <v>29</v>
+      </c>
+      <c r="D10" s="16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="18">
+        <v>88</v>
+      </c>
+      <c r="D11" s="19">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4CE2B3D-AFBC-4BDD-B1BE-7AA2148F6806}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="4" width="19.7265625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="6">
+        <v>76</v>
+      </c>
+      <c r="D2" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="6">
+        <v>45</v>
+      </c>
+      <c r="D3" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="6">
+        <v>41</v>
+      </c>
+      <c r="D4" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="6">
+        <v>57</v>
+      </c>
+      <c r="D5" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="6">
+        <v>63</v>
+      </c>
+      <c r="D6" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="6">
+        <v>35</v>
+      </c>
+      <c r="D7" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="6">
+        <v>23</v>
+      </c>
+      <c r="D8" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="6">
+        <v>52</v>
+      </c>
+      <c r="D9" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="6">
+        <v>29</v>
+      </c>
+      <c r="D10" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="9">
+        <v>88</v>
+      </c>
+      <c r="D11" s="10">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>